<commit_message>
Restock from updated inventry.xlsx — 271 units across 36 SKUs
Notable restocks: ST007, ST010, ST011, ST012, ST013, ST014, and ST015
all gained size coverage. ST014 is no longer fully sold out (1 in XXL).
Total tracked units: 246 → 271.

8 Excel rows still skipped (no catalog entry / photos yet):
  F0001, F0010, ST004, ST008, ST009, ST016, ST017, ST018

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventry.xlsx
+++ b/inventry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sravankumarraparthi/Documents/aark_website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9939958-A675-D849-B366-BEAD5CB530FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{963863A4-77AE-5541-A128-C620DEDF37A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{45664BD4-E25E-D14A-ACD9-9B8700F73003}"/>
+    <workbookView xWindow="2200" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{45664BD4-E25E-D14A-ACD9-9B8700F73003}"/>
   </bookViews>
   <sheets>
     <sheet name="dress" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Dress Code</t>
   </si>
@@ -107,6 +107,57 @@
     <t>ST003</t>
   </si>
   <si>
+    <t>F0002</t>
+  </si>
+  <si>
+    <t>F0013</t>
+  </si>
+  <si>
+    <t>F0012</t>
+  </si>
+  <si>
+    <t>F0005</t>
+  </si>
+  <si>
+    <t>F0004</t>
+  </si>
+  <si>
+    <t>F0003</t>
+  </si>
+  <si>
+    <t>F0009</t>
+  </si>
+  <si>
+    <t>F0006</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>F0001</t>
+  </si>
+  <si>
+    <t>F0010</t>
+  </si>
+  <si>
+    <t>ST004</t>
+  </si>
+  <si>
+    <t>ST015</t>
+  </si>
+  <si>
+    <t>ST013</t>
+  </si>
+  <si>
+    <t>ST007</t>
+  </si>
+  <si>
+    <t>ST008</t>
+  </si>
+  <si>
+    <t>ST009</t>
+  </si>
+  <si>
     <t>ST010</t>
   </si>
   <si>
@@ -116,19 +167,16 @@
     <t>ST012</t>
   </si>
   <si>
-    <t>ST007</t>
+    <t>ST016</t>
+  </si>
+  <si>
+    <t>ST017</t>
+  </si>
+  <si>
+    <t>ST018</t>
   </si>
   <si>
     <t>ST014</t>
-  </si>
-  <si>
-    <t>ST015</t>
-  </si>
-  <si>
-    <t>ST013</t>
-  </si>
-  <si>
-    <t>F0002</t>
   </si>
 </sst>
 </file>
@@ -515,408 +563,1048 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4214986F-0BA5-944F-9122-0962FA07CA67}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
+        <v>3</v>
+      </c>
       <c r="E2" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <v>8</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
       <c r="C3" s="2">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
       <c r="E3" s="2">
         <v>1</v>
       </c>
       <c r="F3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" s="2">
-        <v>2</v>
-      </c>
-      <c r="H3" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
       <c r="C4" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E4" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4" s="2">
         <v>1</v>
       </c>
       <c r="H4" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
       <c r="E6" s="2">
-        <v>1</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="B7" s="2">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
       <c r="E7" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="2">
-        <v>1</v>
-      </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
       <c r="E8" s="2">
-        <v>1</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>2</v>
+      </c>
       <c r="F9" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="2">
-        <v>1</v>
-      </c>
-      <c r="H9" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="B10" s="2">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
+      <c r="B11" s="2">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
       <c r="D11" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G11" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H11" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="B12" s="2">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2</v>
+      </c>
       <c r="D12" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E12" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H12" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="B13" s="2">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2">
+        <v>7</v>
+      </c>
       <c r="E13" s="2">
-        <v>1</v>
-      </c>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2">
+        <v>8</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="B14" s="2">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2">
+        <v>5</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2">
+        <v>10</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0</v>
+      </c>
       <c r="D15" s="2">
-        <v>4</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
       <c r="G15" s="2">
-        <v>3</v>
-      </c>
-      <c r="H15" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1</v>
+      </c>
       <c r="D16" s="2">
         <v>1</v>
       </c>
       <c r="E16" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="2">
-        <v>3</v>
-      </c>
-      <c r="H16" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="B17" s="2">
+        <v>1</v>
+      </c>
       <c r="C17" s="2">
         <v>1</v>
       </c>
       <c r="D17" s="2">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="E17" s="2">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
       <c r="G17" s="2">
-        <v>1</v>
-      </c>
-      <c r="H17" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="H17" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="B18" s="2">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0</v>
+      </c>
+      <c r="E18" s="2">
+        <v>2</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="B19" s="2">
+        <v>2</v>
+      </c>
       <c r="C19" s="2">
-        <v>1</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
+      <c r="H19" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="2"/>
+        <v>30</v>
+      </c>
+      <c r="B20" s="2">
+        <v>1</v>
+      </c>
       <c r="C20" s="2">
-        <v>2</v>
-      </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+        <v>24</v>
+      </c>
+      <c r="B21" s="2">
+        <v>0</v>
+      </c>
+      <c r="C21" s="2">
+        <v>0</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2">
+        <v>1</v>
+      </c>
+      <c r="F21" s="2">
+        <v>1</v>
+      </c>
       <c r="G21" s="2">
         <v>1</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
+        <v>25</v>
+      </c>
+      <c r="B22" s="2">
+        <v>0</v>
+      </c>
+      <c r="C22" s="2">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2">
+        <v>2</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2">
+        <v>5</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
+        <v>29</v>
+      </c>
+      <c r="B23" s="2">
+        <v>0</v>
+      </c>
+      <c r="C23" s="2">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2">
+        <v>0</v>
+      </c>
+      <c r="H23" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
+        <v>33</v>
+      </c>
+      <c r="B24" s="2">
+        <v>0</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0</v>
+      </c>
+      <c r="D24" s="2">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="B25" s="2">
+        <v>3</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0</v>
+      </c>
       <c r="E25" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2">
-        <v>1</v>
-      </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="G25" s="2">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="2">
+        <v>3</v>
+      </c>
+      <c r="C26" s="2">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2">
+        <v>2</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2">
+        <v>2</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="2">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2">
+        <v>0</v>
+      </c>
+      <c r="H27" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="2">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="2">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="2">
+        <v>1</v>
+      </c>
+      <c r="C30" s="2">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2">
+        <v>2</v>
+      </c>
+      <c r="E30" s="2">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" s="2">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2">
+        <v>1</v>
+      </c>
+      <c r="D31" s="2">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" s="2">
+        <v>0</v>
+      </c>
+      <c r="C32" s="2">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2">
+        <v>0</v>
+      </c>
+      <c r="H32" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="2">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2">
+        <v>1</v>
+      </c>
+      <c r="D33" s="2">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2">
+        <v>1</v>
+      </c>
+      <c r="G33" s="2">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" s="2">
+        <v>1</v>
+      </c>
+      <c r="C34" s="2">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2">
+        <v>4</v>
+      </c>
+      <c r="E34" s="2">
+        <v>1</v>
+      </c>
+      <c r="F34" s="2">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35" s="2">
+        <v>1</v>
+      </c>
+      <c r="C35" s="2">
+        <v>0</v>
+      </c>
+      <c r="D35" s="2">
+        <v>2</v>
+      </c>
+      <c r="E35" s="2">
+        <v>1</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2">
+        <v>0</v>
+      </c>
+      <c r="H35" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="2">
+        <v>0</v>
+      </c>
+      <c r="C36" s="2">
+        <v>0</v>
+      </c>
+      <c r="D36" s="2">
+        <v>2</v>
+      </c>
+      <c r="E36" s="2">
+        <v>1</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0</v>
+      </c>
+      <c r="G36" s="2">
+        <v>0</v>
+      </c>
+      <c r="H36" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="2">
+        <v>0</v>
+      </c>
+      <c r="C37" s="2">
+        <v>0</v>
+      </c>
+      <c r="D37" s="2">
+        <v>0</v>
+      </c>
+      <c r="E37" s="2">
+        <v>2</v>
+      </c>
+      <c r="F37" s="2">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2">
+        <v>0</v>
+      </c>
+      <c r="H37" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="2">
+        <v>0</v>
+      </c>
+      <c r="C38" s="2">
+        <v>0</v>
+      </c>
+      <c r="D38" s="2">
+        <v>1</v>
+      </c>
+      <c r="E38" s="2">
+        <v>1</v>
+      </c>
+      <c r="F38" s="2">
+        <v>1</v>
+      </c>
+      <c r="G38" s="2">
+        <v>0</v>
+      </c>
+      <c r="H38" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" s="2">
+        <v>1</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2">
+        <v>0</v>
+      </c>
+      <c r="E39" s="2">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2">
+        <v>0</v>
+      </c>
+      <c r="G39" s="2">
+        <v>1</v>
+      </c>
+      <c r="H39" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" s="2">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2">
+        <v>0</v>
+      </c>
+      <c r="D40" s="2">
+        <v>0</v>
+      </c>
+      <c r="E40" s="2">
+        <v>0</v>
+      </c>
+      <c r="F40" s="2">
+        <v>0</v>
+      </c>
+      <c r="G40" s="2">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Inventory update via admin — 2026-05-13T03:35:38Z
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventry.xlsx
+++ b/inventry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sravankumarraparthi/Documents/aark_website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{963863A4-77AE-5541-A128-C620DEDF37A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B69832-D4F8-9D46-A25C-44E8F6C97FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2200" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{45664BD4-E25E-D14A-ACD9-9B8700F73003}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Dress Code</t>
   </si>
@@ -68,12 +68,6 @@
     <t>SC003</t>
   </si>
   <si>
-    <t>SC004</t>
-  </si>
-  <si>
-    <t>SC005</t>
-  </si>
-  <si>
     <t>SC006</t>
   </si>
   <si>
@@ -83,9 +77,6 @@
     <t>SC008</t>
   </si>
   <si>
-    <t>SC009</t>
-  </si>
-  <si>
     <t>SC010</t>
   </si>
   <si>
@@ -132,12 +123,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>F0001</t>
-  </si>
-  <si>
-    <t>F0010</t>
   </si>
   <si>
     <t>ST004</t>
@@ -589,7 +574,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -684,7 +669,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="2">
         <v>0</v>
@@ -693,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -707,7 +692,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2">
         <v>0</v>
@@ -719,7 +704,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -736,7 +721,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -745,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -756,22 +741,22 @@
         <v>0</v>
       </c>
       <c r="C8" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8" s="2">
         <v>0</v>
       </c>
       <c r="H8" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -782,22 +767,22 @@
         <v>0</v>
       </c>
       <c r="C9" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E9" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="2">
         <v>0</v>
       </c>
       <c r="H9" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -808,10 +793,10 @@
         <v>0</v>
       </c>
       <c r="C10" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E10" s="2">
         <v>0</v>
@@ -823,7 +808,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -834,65 +819,65 @@
         <v>0</v>
       </c>
       <c r="C11" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D11" s="2">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2">
         <v>3</v>
       </c>
-      <c r="E11" s="2">
-        <v>4</v>
-      </c>
       <c r="F11" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2">
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E12" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="2">
         <v>0</v>
       </c>
       <c r="H12" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" s="2">
         <v>1</v>
       </c>
       <c r="D13" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
@@ -901,47 +886,47 @@
         <v>0</v>
       </c>
       <c r="H13" s="2">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B14" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2">
         <v>0</v>
       </c>
       <c r="E14" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" s="2">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B15" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C15" s="2">
         <v>0</v>
       </c>
       <c r="D15" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="2">
         <v>0</v>
@@ -953,21 +938,21 @@
         <v>0</v>
       </c>
       <c r="H15" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
       </c>
       <c r="D16" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="2">
         <v>0</v>
@@ -984,54 +969,54 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B17" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" s="2">
         <v>1</v>
       </c>
       <c r="F17" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B18" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
       </c>
       <c r="D18" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E18" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="2">
         <v>0</v>
       </c>
       <c r="H18" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -1039,16 +1024,16 @@
         <v>26</v>
       </c>
       <c r="B19" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C19" s="2">
         <v>0</v>
       </c>
       <c r="D19" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -1057,18 +1042,18 @@
         <v>0</v>
       </c>
       <c r="H19" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B20" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="2">
         <v>0</v>
@@ -1077,56 +1062,56 @@
         <v>0</v>
       </c>
       <c r="F20" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20" s="2">
         <v>0</v>
       </c>
       <c r="H20" s="2">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C21" s="2">
         <v>0</v>
       </c>
       <c r="D21" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B22" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
       </c>
       <c r="D22" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E22" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2">
         <v>1</v>
@@ -1135,7 +1120,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -1143,13 +1128,13 @@
         <v>29</v>
       </c>
       <c r="B23" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C23" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="2">
         <v>1</v>
@@ -1161,24 +1146,24 @@
         <v>0</v>
       </c>
       <c r="H23" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B24" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D24" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="2">
         <v>0</v>
@@ -1187,85 +1172,85 @@
         <v>0</v>
       </c>
       <c r="H24" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B25" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C25" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E25" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="2">
         <v>0</v>
       </c>
       <c r="H25" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B26" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C26" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E26" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="2">
         <v>0</v>
       </c>
       <c r="H26" s="2">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="B27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="2">
         <v>0</v>
       </c>
       <c r="F27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" s="2">
         <v>0</v>
       </c>
       <c r="H27" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -1273,25 +1258,25 @@
         <v>34</v>
       </c>
       <c r="B28" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C28" s="2">
         <v>1</v>
       </c>
       <c r="D28" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" s="2">
         <v>0</v>
       </c>
       <c r="H28" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -1302,10 +1287,10 @@
         <v>1</v>
       </c>
       <c r="C29" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E29" s="2">
         <v>1</v>
@@ -1317,7 +1302,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -1354,10 +1339,10 @@
         <v>0</v>
       </c>
       <c r="C31" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E31" s="2">
         <v>1</v>
@@ -1369,7 +1354,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -1383,10 +1368,10 @@
         <v>0</v>
       </c>
       <c r="D32" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F32" s="2">
         <v>0</v>
@@ -1395,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -1406,13 +1391,13 @@
         <v>0</v>
       </c>
       <c r="C33" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" s="2">
         <v>1</v>
@@ -1421,7 +1406,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -1432,22 +1417,22 @@
         <v>1</v>
       </c>
       <c r="C34" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E34" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" s="2">
         <v>0</v>
       </c>
       <c r="G34" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -1461,10 +1446,10 @@
         <v>0</v>
       </c>
       <c r="D35" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E35" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2">
         <v>0</v>
@@ -1473,138 +1458,58 @@
         <v>0</v>
       </c>
       <c r="H35" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B36" s="2">
-        <v>0</v>
-      </c>
-      <c r="C36" s="2">
-        <v>0</v>
-      </c>
-      <c r="D36" s="2">
-        <v>2</v>
-      </c>
-      <c r="E36" s="2">
-        <v>1</v>
-      </c>
-      <c r="F36" s="2">
-        <v>0</v>
-      </c>
-      <c r="G36" s="2">
-        <v>0</v>
-      </c>
-      <c r="H36" s="2">
-        <v>3</v>
-      </c>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B37" s="2">
-        <v>0</v>
-      </c>
-      <c r="C37" s="2">
-        <v>0</v>
-      </c>
-      <c r="D37" s="2">
-        <v>0</v>
-      </c>
-      <c r="E37" s="2">
-        <v>2</v>
-      </c>
-      <c r="F37" s="2">
-        <v>0</v>
-      </c>
-      <c r="G37" s="2">
-        <v>0</v>
-      </c>
-      <c r="H37" s="2">
-        <v>2</v>
-      </c>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B38" s="2">
-        <v>0</v>
-      </c>
-      <c r="C38" s="2">
-        <v>0</v>
-      </c>
-      <c r="D38" s="2">
-        <v>1</v>
-      </c>
-      <c r="E38" s="2">
-        <v>1</v>
-      </c>
-      <c r="F38" s="2">
-        <v>1</v>
-      </c>
-      <c r="G38" s="2">
-        <v>0</v>
-      </c>
-      <c r="H38" s="2">
-        <v>3</v>
-      </c>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B39" s="2">
-        <v>1</v>
-      </c>
-      <c r="C39" s="2">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2">
-        <v>0</v>
-      </c>
-      <c r="E39" s="2">
-        <v>0</v>
-      </c>
-      <c r="F39" s="2">
-        <v>0</v>
-      </c>
-      <c r="G39" s="2">
-        <v>1</v>
-      </c>
-      <c r="H39" s="2">
-        <v>3</v>
-      </c>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B40" s="2">
-        <v>1</v>
-      </c>
-      <c r="C40" s="2">
-        <v>0</v>
-      </c>
-      <c r="D40" s="2">
-        <v>0</v>
-      </c>
-      <c r="E40" s="2">
-        <v>0</v>
-      </c>
-      <c r="F40" s="2">
-        <v>0</v>
-      </c>
-      <c r="G40" s="2">
-        <v>0</v>
-      </c>
-      <c r="H40" s="2">
-        <v>1</v>
-      </c>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>